<commit_message>
feat: update default tags and map project tags from schedule
</commit_message>
<xml_diff>
--- a/data/import_ready/projects.xlsx
+++ b/data/import_ready/projects.xlsx
@@ -475,7 +475,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>EdTech</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -508,11 +508,7 @@
           <t>@user_582</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>Образовательный</t>
@@ -542,11 +538,7 @@
           <t>@user_154</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Образовательный</t>
@@ -578,11 +570,7 @@
           <t>@user_583</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Образовательный</t>
@@ -613,7 +601,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>EdTech, NLP, Agents</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -648,11 +636,7 @@
           <t>@user_341</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>Образовательный</t>
@@ -680,11 +664,7 @@
           <t>@user_058</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -707,11 +687,7 @@
           <t>@user_336</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -734,11 +710,7 @@
           <t>@user_042</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -766,11 +738,7 @@
           <t>@user_152</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -799,7 +767,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>CV, Recsys</t>
         </is>
       </c>
     </row>
@@ -827,11 +795,7 @@
           <t>@user_584</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -858,7 +822,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>NLP, Agents, ASR</t>
         </is>
       </c>
     </row>
@@ -885,11 +849,7 @@
           <t>@user_586</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -916,7 +876,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>Recsys</t>
         </is>
       </c>
     </row>
@@ -943,7 +903,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>TimeSeries, RL, Industrial</t>
         </is>
       </c>
     </row>
@@ -972,11 +932,7 @@
           <t>@user_587</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1000,11 +956,7 @@
           <t>@user_320</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1031,11 +983,7 @@
           <t>@user_208</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1062,7 +1010,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>CV, NLP, Industrial</t>
         </is>
       </c>
     </row>
@@ -1089,11 +1037,7 @@
           <t>@user_590</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1118,11 +1062,7 @@
           <t>@user_356</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1151,7 +1091,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>Agents</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1120,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>Recsys, NLP, Agents, AgriTech</t>
         </is>
       </c>
     </row>
@@ -1206,11 +1146,7 @@
           <t>@user_591</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1237,7 +1173,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>CV</t>
         </is>
       </c>
     </row>
@@ -1267,11 +1203,7 @@
           <t>@user_310</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1297,7 +1229,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>NLP, Agents, ASR, TTS</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1256,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>CV, NLP, Agents</t>
         </is>
       </c>
     </row>
@@ -1349,11 +1281,7 @@
           <t>@user_072</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1379,11 +1307,7 @@
           <t>@user_593</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1409,11 +1333,7 @@
           <t>@user_116</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1436,11 +1356,7 @@
           <t>@user_594</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1463,11 +1379,7 @@
           <t>@user_597</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1497,7 +1409,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>NLP</t>
         </is>
       </c>
     </row>
@@ -1524,11 +1436,7 @@
           <t>@user_598</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1551,11 +1459,7 @@
           <t>@user_300</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1579,11 +1483,7 @@
           <t>@user_161</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1611,7 +1511,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>MedTech</t>
         </is>
       </c>
     </row>
@@ -1637,11 +1537,7 @@
           <t>@user_343</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1667,11 +1563,7 @@
           <t>@user_392</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1696,11 +1588,7 @@
           <t>@user_218</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1724,11 +1612,7 @@
           <t>@user_184</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1751,11 +1635,7 @@
           <t>@user_043</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1779,11 +1659,7 @@
           <t>@user_601</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1807,11 +1683,7 @@
           <t>@user_222</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1834,11 +1706,7 @@
           <t>@user_412</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1861,11 +1729,7 @@
           <t>@user_142</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1888,11 +1752,7 @@
           <t>@user_602</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1917,11 +1777,7 @@
           <t>@user_411</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1946,11 +1802,7 @@
           <t>@user_306</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1975,11 +1827,7 @@
           <t>@user_603</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2006,11 +1854,7 @@
           <t>@user_200</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2039,7 +1883,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Научный</t>
+          <t>CV</t>
         </is>
       </c>
     </row>
@@ -2064,11 +1908,7 @@
           <t>@user_229</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2091,11 +1931,7 @@
           <t>@user_050</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2121,11 +1957,7 @@
           <t>@user_604</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2148,11 +1980,7 @@
           <t>@user_165</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2178,11 +2006,7 @@
           <t>@user_221</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2205,11 +2029,7 @@
           <t>@user_114</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2233,11 +2053,7 @@
           <t>@user_304</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2262,11 +2078,7 @@
           <t>@user_064</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2292,11 +2104,7 @@
           <t>@user_125</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2322,11 +2130,7 @@
           <t>@user_003</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2349,11 +2153,7 @@
           <t>@user_375</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2378,11 +2178,7 @@
           <t>@user_295</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2405,11 +2201,7 @@
           <t>@user_318</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2433,11 +2225,7 @@
           <t>@user_605</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2460,11 +2248,7 @@
           <t>@user_606</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2490,11 +2274,7 @@
           <t>@user_607</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2517,11 +2297,7 @@
           <t>@user_608</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2546,11 +2322,7 @@
           <t>@user_273</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2575,11 +2347,7 @@
           <t>@user_447</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2604,11 +2372,7 @@
           <t>@user_201</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2634,11 +2398,7 @@
           <t>@user_420</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2661,11 +2421,7 @@
           <t>@user_395</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2691,11 +2447,7 @@
           <t>@user_260</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2718,11 +2470,7 @@
           <t>@user_180</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2745,11 +2493,7 @@
           <t>@user_609</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2775,11 +2519,7 @@
           <t>@user_610</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2803,11 +2543,7 @@
           <t>@user_352</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2832,11 +2568,7 @@
           <t>@user_004</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2861,11 +2593,7 @@
           <t>@user_020</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2891,11 +2619,7 @@
           <t>@user_053</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2920,11 +2644,7 @@
           <t>@user_612</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2948,11 +2668,7 @@
           <t>@user_013</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2975,11 +2691,7 @@
           <t>@user_178</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3002,11 +2714,7 @@
           <t>@user_030</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3031,11 +2739,7 @@
           <t>@user_614</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3059,11 +2763,7 @@
           <t>@user_245</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3087,11 +2787,7 @@
           <t>@user_027</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3116,11 +2812,7 @@
           <t>@user_206</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3146,11 +2838,7 @@
           <t>@user_073</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3175,11 +2863,7 @@
           <t>@user_402</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3205,11 +2889,7 @@
           <t>@user_214</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3232,11 +2912,7 @@
           <t>@user_302</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3261,11 +2937,7 @@
           <t>@user_405</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3288,11 +2960,7 @@
           <t>@user_239</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3318,11 +2986,7 @@
           <t>@user_453</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3348,11 +3012,7 @@
           <t>@user_092</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3378,11 +3038,7 @@
           <t>@user_616</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3408,11 +3064,7 @@
           <t>@user_282</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3435,11 +3087,7 @@
           <t>@user_006</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3465,11 +3113,7 @@
           <t>@user_279</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3494,11 +3138,7 @@
           <t>@user_291</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3524,11 +3164,7 @@
           <t>@user_205</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3552,11 +3188,7 @@
           <t>@user_617</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3580,11 +3212,7 @@
           <t>@user_298</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3610,11 +3238,7 @@
           <t>@user_434</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3641,11 +3265,7 @@
           <t>@user_014</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3668,11 +3288,7 @@
           <t>@user_618</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3695,11 +3311,7 @@
           <t>@user_619</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3723,11 +3335,7 @@
           <t>@user_380</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3750,11 +3358,7 @@
           <t>@user_002</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3777,11 +3381,7 @@
           <t>@user_620</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3806,11 +3406,7 @@
           <t>@user_436</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3834,11 +3430,7 @@
           <t>@user_621</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3861,11 +3453,7 @@
           <t>@user_059</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3889,11 +3477,7 @@
           <t>@user_241</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3922,7 +3506,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>CV</t>
         </is>
       </c>
     </row>
@@ -3949,11 +3533,7 @@
           <t>@user_622</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3978,11 +3558,7 @@
           <t>@user_067</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4008,11 +3584,7 @@
           <t>@user_079</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4035,11 +3607,7 @@
           <t>@user_408</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4065,7 +3633,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>NLP</t>
         </is>
       </c>
     </row>
@@ -4092,11 +3660,7 @@
           <t>@user_314</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4120,11 +3684,7 @@
           <t>@user_140</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4148,11 +3708,7 @@
           <t>@user_624</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4175,11 +3731,7 @@
           <t>@user_071</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4202,11 +3754,7 @@
           <t>@user_262</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4229,11 +3777,7 @@
           <t>@user_136</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4260,11 +3804,7 @@
           <t>@user_625</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4289,7 +3829,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>CV, NLP, ASR, TTS</t>
         </is>
       </c>
     </row>
@@ -4314,11 +3854,7 @@
           <t>@user_090</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4341,11 +3877,7 @@
           <t>@user_626</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4369,11 +3901,7 @@
           <t>@user_627</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4396,11 +3924,7 @@
           <t>@user_226</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4427,7 +3951,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>Agents, NLP</t>
         </is>
       </c>
     </row>
@@ -4457,11 +3981,7 @@
           <t>@user_363</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -4487,11 +4007,7 @@
           <t>@user_406</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -4518,11 +4034,7 @@
           <t>@user_452</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -4547,11 +4059,7 @@
           <t>@user_628</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -4576,11 +4084,7 @@
           <t>@user_238</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4606,11 +4110,7 @@
           <t>@user_127</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -4635,11 +4135,7 @@
           <t>@user_085</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -4662,11 +4158,7 @@
           <t>@user_629</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -4694,7 +4186,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>CV, NLP</t>
         </is>
       </c>
     </row>
@@ -4721,11 +4213,7 @@
           <t>@user_487</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -4750,11 +4238,7 @@
           <t>@user_631</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -4780,11 +4264,7 @@
           <t>@user_632</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -4807,11 +4287,7 @@
           <t>@user_400</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -4837,11 +4313,7 @@
           <t>@user_633</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -4865,11 +4337,7 @@
           <t>@user_416</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -4894,7 +4362,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>NLP, ML</t>
         </is>
       </c>
     </row>
@@ -4921,11 +4389,7 @@
           <t>@user_636</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -4951,11 +4415,7 @@
           <t>@user_227</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -4978,11 +4438,7 @@
           <t>@user_364</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -5005,11 +4461,7 @@
           <t>@user_081</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -5035,11 +4487,7 @@
           <t>@user_288</t>
         </is>
       </c>
-      <c r="E160" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -5062,11 +4510,7 @@
           <t>@user_638</t>
         </is>
       </c>
-      <c r="E161" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -5089,11 +4533,7 @@
           <t>@user_138</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -5121,7 +4561,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>Recsys</t>
         </is>
       </c>
     </row>
@@ -5146,11 +4586,7 @@
           <t>@user_089</t>
         </is>
       </c>
-      <c r="E164" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -5174,11 +4610,7 @@
           <t>@user_435</t>
         </is>
       </c>
-      <c r="E165" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -5203,7 +4635,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>Agents, NLP</t>
         </is>
       </c>
     </row>
@@ -5229,11 +4661,7 @@
           <t>@user_309</t>
         </is>
       </c>
-      <c r="E167" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -5258,11 +4686,7 @@
           <t>@user_213</t>
         </is>
       </c>
-      <c r="E168" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -5287,7 +4711,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>Agents, EdTech, Recsys, NLP</t>
         </is>
       </c>
     </row>
@@ -5314,7 +4738,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>NLP</t>
         </is>
       </c>
     </row>
@@ -5341,11 +4765,7 @@
           <t>@user_193</t>
         </is>
       </c>
-      <c r="E171" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -5372,7 +4792,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>NLP, ML</t>
         </is>
       </c>
     </row>
@@ -5397,11 +4817,7 @@
           <t>@user_076</t>
         </is>
       </c>
-      <c r="E173" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -5426,11 +4842,7 @@
           <t>@user_482</t>
         </is>
       </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -5455,11 +4867,7 @@
           <t>@user_422</t>
         </is>
       </c>
-      <c r="E175" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -5484,7 +4892,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>Recsys</t>
         </is>
       </c>
     </row>
@@ -5512,11 +4920,7 @@
           <t>@user_640</t>
         </is>
       </c>
-      <c r="E177" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -5539,11 +4943,7 @@
           <t>@user_641</t>
         </is>
       </c>
-      <c r="E178" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -5566,11 +4966,7 @@
           <t>@user_388</t>
         </is>
       </c>
-      <c r="E179" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -5594,11 +4990,7 @@
           <t>@user_243</t>
         </is>
       </c>
-      <c r="E180" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -5621,11 +5013,7 @@
           <t>@user_644</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -5652,11 +5040,7 @@
           <t>@user_317</t>
         </is>
       </c>
-      <c r="E182" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -5682,11 +5066,7 @@
           <t>@user_270</t>
         </is>
       </c>
-      <c r="E183" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -5711,11 +5091,7 @@
           <t>@user_439</t>
         </is>
       </c>
-      <c r="E184" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -5745,7 +5121,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>Industrial, NLP</t>
         </is>
       </c>
     </row>
@@ -5771,11 +5147,7 @@
           <t>@user_645</t>
         </is>
       </c>
-      <c r="E186" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -5800,11 +5172,7 @@
           <t>@user_266</t>
         </is>
       </c>
-      <c r="E187" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -5829,11 +5197,7 @@
           <t>@user_024</t>
         </is>
       </c>
-      <c r="E188" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -5856,11 +5220,7 @@
           <t>@user_647</t>
         </is>
       </c>
-      <c r="E189" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -5885,11 +5245,7 @@
           <t>@user_086</t>
         </is>
       </c>
-      <c r="E190" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -5913,11 +5269,7 @@
           <t>@user_473</t>
         </is>
       </c>
-      <c r="E191" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -5940,11 +5292,7 @@
           <t>@user_649</t>
         </is>
       </c>
-      <c r="E192" t="inlineStr">
-        <is>
-          <t>Другое</t>
-        </is>
-      </c>
+      <c r="E192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -5969,7 +5317,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Другое</t>
+          <t>Industrial</t>
         </is>
       </c>
     </row>
@@ -5994,11 +5342,7 @@
           <t>@user_255</t>
         </is>
       </c>
-      <c r="E194" t="inlineStr">
-        <is>
-          <t>Другое</t>
-        </is>
-      </c>
+      <c r="E194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -6023,11 +5367,7 @@
           <t>@user_312</t>
         </is>
       </c>
-      <c r="E195" t="inlineStr">
-        <is>
-          <t>Другое</t>
-        </is>
-      </c>
+      <c r="E195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -6055,7 +5395,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>EdTech, NLP</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -6090,11 +5430,7 @@
           <t>@user_650</t>
         </is>
       </c>
-      <c r="E197" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
+      <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr">
         <is>
           <t>Образовательный</t>
@@ -6126,11 +5462,7 @@
           <t>@expert_249</t>
         </is>
       </c>
-      <c r="E198" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
+      <c r="E198" t="inlineStr"/>
       <c r="F198" t="inlineStr">
         <is>
           <t>Образовательный</t>
@@ -6158,11 +5490,7 @@
           <t>@user_264</t>
         </is>
       </c>
-      <c r="E199" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
+      <c r="E199" t="inlineStr"/>
       <c r="F199" t="inlineStr">
         <is>
           <t>Образовательный</t>
@@ -6190,11 +5518,7 @@
           <t>@expert_193</t>
         </is>
       </c>
-      <c r="E200" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
+      <c r="E200" t="inlineStr"/>
       <c r="F200" t="inlineStr">
         <is>
           <t>Образовательный</t>
@@ -6225,11 +5549,7 @@
           <t>@user_009</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr">
-        <is>
-          <t>Education</t>
-        </is>
-      </c>
+      <c r="E201" t="inlineStr"/>
       <c r="F201" t="inlineStr">
         <is>
           <t>Образовательный</t>
@@ -6259,7 +5579,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>EdTech</t>
         </is>
       </c>
     </row>
@@ -6289,7 +5609,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>NLP, Agents</t>
         </is>
       </c>
     </row>
@@ -6315,11 +5635,7 @@
           <t>@user_651</t>
         </is>
       </c>
-      <c r="E204" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -6346,7 +5662,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>NLP, EdTech</t>
         </is>
       </c>
     </row>
@@ -6375,7 +5691,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>EdTech, NLP</t>
         </is>
       </c>
     </row>
@@ -6402,7 +5718,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Стартап</t>
+          <t>NLP, RL</t>
         </is>
       </c>
     </row>
@@ -6427,11 +5743,7 @@
           <t>@user_070</t>
         </is>
       </c>
-      <c r="E208" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -6456,11 +5768,7 @@
           <t>@user_045</t>
         </is>
       </c>
-      <c r="E209" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -6483,11 +5791,7 @@
           <t>@user_653</t>
         </is>
       </c>
-      <c r="E210" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -6514,11 +5818,7 @@
           <t>@user_035</t>
         </is>
       </c>
-      <c r="E211" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -6543,11 +5843,7 @@
           <t>@user_335</t>
         </is>
       </c>
-      <c r="E212" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -6571,11 +5867,7 @@
           <t>@user_654</t>
         </is>
       </c>
-      <c r="E213" t="inlineStr">
-        <is>
-          <t>Стартап</t>
-        </is>
-      </c>
+      <c r="E213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -6599,11 +5891,7 @@
           <t>@expert_067</t>
         </is>
       </c>
-      <c r="E214" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -6626,11 +5914,7 @@
           <t>@user_170</t>
         </is>
       </c>
-      <c r="E215" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -6653,11 +5937,7 @@
           <t>@user_358</t>
         </is>
       </c>
-      <c r="E216" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -6685,11 +5965,7 @@
           <t>@user_386</t>
         </is>
       </c>
-      <c r="E217" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -6712,11 +5988,7 @@
           <t>@expert_202</t>
         </is>
       </c>
-      <c r="E218" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -6739,11 +6011,7 @@
           <t>@expert_115</t>
         </is>
       </c>
-      <c r="E219" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -6767,11 +6035,7 @@
           <t>@user_359</t>
         </is>
       </c>
-      <c r="E220" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -6795,11 +6059,7 @@
           <t>@user_481</t>
         </is>
       </c>
-      <c r="E221" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -6825,11 +6085,7 @@
           <t>@user_381</t>
         </is>
       </c>
-      <c r="E222" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -6853,11 +6109,7 @@
           <t>@user_237</t>
         </is>
       </c>
-      <c r="E223" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -6881,11 +6133,7 @@
           <t>@user_060</t>
         </is>
       </c>
-      <c r="E224" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -6909,11 +6157,7 @@
           <t>@expert_212</t>
         </is>
       </c>
-      <c r="E225" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -6936,11 +6180,7 @@
           <t>@user_203</t>
         </is>
       </c>
-      <c r="E226" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -6963,11 +6203,7 @@
           <t>@user_378</t>
         </is>
       </c>
-      <c r="E227" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -6990,11 +6226,7 @@
           <t>@user_431</t>
         </is>
       </c>
-      <c r="E228" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -7019,11 +6251,7 @@
           <t>@user_377</t>
         </is>
       </c>
-      <c r="E229" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -7050,11 +6278,7 @@
           <t>@user_467</t>
         </is>
       </c>
-      <c r="E230" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -7078,11 +6302,7 @@
           <t>@user_656</t>
         </is>
       </c>
-      <c r="E231" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -7107,7 +6327,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>NLP</t>
         </is>
       </c>
     </row>
@@ -7134,11 +6354,7 @@
           <t>@user_353</t>
         </is>
       </c>
-      <c r="E233" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -7161,11 +6377,7 @@
           <t>@user_657</t>
         </is>
       </c>
-      <c r="E234" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -7190,7 +6402,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>NLP</t>
         </is>
       </c>
     </row>
@@ -7218,11 +6430,7 @@
           <t>@user_319</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -7248,11 +6456,7 @@
           <t>@expert_097</t>
         </is>
       </c>
-      <c r="E237" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -7277,7 +6481,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>CV</t>
         </is>
       </c>
     </row>
@@ -7307,11 +6511,7 @@
           <t>@expert_169</t>
         </is>
       </c>
-      <c r="E239" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -7334,11 +6534,7 @@
           <t>@user_272</t>
         </is>
       </c>
-      <c r="E240" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -7362,11 +6558,7 @@
           <t>@user_414</t>
         </is>
       </c>
-      <c r="E241" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -7392,11 +6584,7 @@
           <t>@user_658</t>
         </is>
       </c>
-      <c r="E242" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -7420,11 +6608,7 @@
           <t>@user_062</t>
         </is>
       </c>
-      <c r="E243" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -7450,7 +6634,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>FinTech</t>
         </is>
       </c>
     </row>
@@ -7479,11 +6663,7 @@
           <t>@user_028</t>
         </is>
       </c>
-      <c r="E245" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -7511,7 +6691,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>Industrial, RAG, NLP, Agents</t>
         </is>
       </c>
     </row>
@@ -7538,11 +6718,7 @@
           <t>@user_391</t>
         </is>
       </c>
-      <c r="E247" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -7567,11 +6743,7 @@
           <t>@expert_156</t>
         </is>
       </c>
-      <c r="E248" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -7594,11 +6766,7 @@
           <t>@user_464</t>
         </is>
       </c>
-      <c r="E249" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -7622,11 +6790,7 @@
           <t>@user_660</t>
         </is>
       </c>
-      <c r="E250" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -7652,7 +6816,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>Agents, NLP</t>
         </is>
       </c>
     </row>
@@ -7680,11 +6844,7 @@
           <t>@user_278</t>
         </is>
       </c>
-      <c r="E252" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -7710,11 +6870,7 @@
           <t>@user_459</t>
         </is>
       </c>
-      <c r="E253" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -7738,11 +6894,7 @@
           <t>@user_215</t>
         </is>
       </c>
-      <c r="E254" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -7766,11 +6918,7 @@
           <t>@user_194</t>
         </is>
       </c>
-      <c r="E255" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -7795,11 +6943,7 @@
           <t>@user_007</t>
         </is>
       </c>
-      <c r="E256" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -7822,11 +6966,7 @@
           <t>@user_311</t>
         </is>
       </c>
-      <c r="E257" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -7852,11 +6992,7 @@
           <t>@user_181</t>
         </is>
       </c>
-      <c r="E258" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -7883,7 +7019,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>Recsys</t>
         </is>
       </c>
     </row>
@@ -7909,11 +7045,7 @@
           <t>@user_189</t>
         </is>
       </c>
-      <c r="E260" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -7939,11 +7071,7 @@
           <t>@expert_023</t>
         </is>
       </c>
-      <c r="E261" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -7966,11 +7094,7 @@
           <t>@user_463</t>
         </is>
       </c>
-      <c r="E262" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -7998,7 +7122,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>FinTech</t>
         </is>
       </c>
     </row>
@@ -8031,7 +7155,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>FinTech</t>
         </is>
       </c>
     </row>
@@ -8058,11 +7182,7 @@
           <t>@user_230</t>
         </is>
       </c>
-      <c r="E265" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -8088,11 +7208,7 @@
           <t>@user_662</t>
         </is>
       </c>
-      <c r="E266" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -8115,11 +7231,7 @@
           <t>@user_155</t>
         </is>
       </c>
-      <c r="E267" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -8146,11 +7258,7 @@
           <t>@user_348</t>
         </is>
       </c>
-      <c r="E268" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -8175,11 +7283,7 @@
           <t>@user_121</t>
         </is>
       </c>
-      <c r="E269" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -8203,11 +7307,7 @@
           <t>@expert_029</t>
         </is>
       </c>
-      <c r="E270" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -8230,11 +7330,7 @@
           <t>@user_268</t>
         </is>
       </c>
-      <c r="E271" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -8258,11 +7354,7 @@
           <t>@expert_205</t>
         </is>
       </c>
-      <c r="E272" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -8285,11 +7377,7 @@
           <t>@user_664</t>
         </is>
       </c>
-      <c r="E273" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -8313,11 +7401,7 @@
           <t>@user_443</t>
         </is>
       </c>
-      <c r="E274" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -8342,11 +7426,7 @@
           <t>@user_665</t>
         </is>
       </c>
-      <c r="E275" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -8373,11 +7453,7 @@
           <t>@user_666</t>
         </is>
       </c>
-      <c r="E276" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -8402,11 +7478,7 @@
           <t>@user_204</t>
         </is>
       </c>
-      <c r="E277" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -8431,11 +7503,7 @@
           <t>@user_261</t>
         </is>
       </c>
-      <c r="E278" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -8458,11 +7526,7 @@
           <t>@user_277</t>
         </is>
       </c>
-      <c r="E279" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -8485,11 +7549,7 @@
           <t>@user_470</t>
         </is>
       </c>
-      <c r="E280" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -8514,11 +7574,7 @@
           <t>@user_236</t>
         </is>
       </c>
-      <c r="E281" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -8541,11 +7597,7 @@
           <t>@user_190</t>
         </is>
       </c>
-      <c r="E282" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -8568,11 +7620,7 @@
           <t>@user_134</t>
         </is>
       </c>
-      <c r="E283" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -8597,7 +7645,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>NLP</t>
         </is>
       </c>
     </row>
@@ -8626,7 +7674,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>Recsys, Industrial</t>
         </is>
       </c>
     </row>
@@ -8654,7 +7702,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Индустриальный</t>
+          <t>Backend, NLP</t>
         </is>
       </c>
     </row>
@@ -8682,11 +7730,7 @@
           <t>@user_437</t>
         </is>
       </c>
-      <c r="E287" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -8711,11 +7755,7 @@
           <t>@user_486</t>
         </is>
       </c>
-      <c r="E288" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -8740,11 +7780,7 @@
           <t>@user_340</t>
         </is>
       </c>
-      <c r="E289" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -8769,11 +7805,7 @@
           <t>@user_430</t>
         </is>
       </c>
-      <c r="E290" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -8800,11 +7832,7 @@
           <t>@user_672</t>
         </is>
       </c>
-      <c r="E291" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -8828,11 +7856,7 @@
           <t>@user_259</t>
         </is>
       </c>
-      <c r="E292" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -8856,11 +7880,7 @@
           <t>@user_157</t>
         </is>
       </c>
-      <c r="E293" t="inlineStr">
-        <is>
-          <t>Индустриальный</t>
-        </is>
-      </c>
+      <c r="E293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -8885,11 +7905,7 @@
           <t>@user_370</t>
         </is>
       </c>
-      <c r="E294" t="inlineStr">
-        <is>
-          <t>Научный</t>
-        </is>
-      </c>
+      <c r="E294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -8914,7 +7930,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Другое</t>
+          <t>Recsys, NLP</t>
         </is>
       </c>
     </row>

</xml_diff>